<commit_message>
test(data): certify controlled local replay pack
</commit_message>
<xml_diff>
--- a/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
+++ b/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="Rc4c5bcc5c29c4e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="Rf96429bcce6144c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="R6e30f1ef23c9458b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="R3eb48113a483486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="Rae408795cca54a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="Rb75fe10c493544b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="R81288d98edce4ddc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="R870bf78e6bb8465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R32fd5d83ac5d489e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="R0198cfdc4194453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="Rce398ca90a7d4be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R955ec46df0a34345"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="R04b6215bcdba44b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="R85be943f034a412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="R5e057976c5744762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="Rbf2198b3cfb048da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="Rf26e28fc35ee48f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="Rc94a930d94e74d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="Rcf86e6669bfa4898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="R4be72473a09147d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="R72c1ce6851f34a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="Rd9fa693efc0c4dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="R88dbd92e23ae4d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="Rf22c1128ace64030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="R261e0bd7c5f8495f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R441d130d4dc342b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="Rb8226e95fb5d4f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="R5b1a831b8ea04dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R18a4068ec0e54ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="Rd5585572708242ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="R8b62ffb6494147ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="Rf604819390f64536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="Re8d240c01e3d4a66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="R3c56eb7f14b14a9c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -373,23 +373,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TAccounts" displayName="TAccounts" ref="A3:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:F23"/>
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TAccounts" displayName="TAccounts" ref="A3:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:E25"/>
+  <x:tableColumns count="5">
     <x:tableColumn id="1" name="Username"/>
     <x:tableColumn id="2" name="Hidden Auth Email"/>
-    <x:tableColumn id="3" name="Role"/>
+    <x:tableColumn id="3" name="Role Grants"/>
     <x:tableColumn id="4" name="User ID"/>
-    <x:tableColumn id="5" name="Local QA Password"/>
-    <x:tableColumn id="6" name="Password Guard"/>
+    <x:tableColumn id="5" name="Credential Source"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TProfiles" displayName="TProfiles" ref="A3:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:F23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TProfiles" displayName="TProfiles" ref="A3:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:F25"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="User ID"/>
     <x:tableColumn id="2" name="Username"/>
@@ -700,7 +699,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14.779999732971191" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -756,10 +755,10 @@
         <x:v>QA password</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>Password</x:v>
+        <x:v>OPERATOR SUPPLIED</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>Allowed only when environment guard proves local</x:v>
+        <x:v>Required through fail-closed environment loading; never stored in this package</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -824,7 +823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bf8b043776542e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52dbd542a6c4958"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -988,7 +987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb77f492cfe94302"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48902a7d58e447b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1127,7 +1126,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46db0c8d12044895"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e3466ada3c94389"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1351,7 +1350,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2fb633d4e3f4bfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e7693d0c0cd41e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1578,7 +1577,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf50b8dafc93b4c65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13bc69a397f74d99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1648,19 +1647,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18" t="str">
-        <x:v>Profiles</x:v>
+        <x:v>Accounts</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>Role</x:v>
+        <x:v>Role Grants</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>enum</x:v>
+        <x:v>enum list</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Boundary aware</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>One of admin/planner/supervisor/inspector</x:v>
+        <x:v>Canonical role grant(s), or none for the no-workspace refusal persona</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1738,7 +1737,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb91253eaf2d43e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954ad43bdd244055"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1819,7 +1818,7 @@
         <x:v>Auth users</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>Upsert 20 deterministic local identities</x:v>
+        <x:v>Upsert 22 deterministic local identities</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>15</x:v>
@@ -1930,7 +1929,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1341e5578c9a48f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f31b32a3fae4019"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1939,7 +1938,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="7.670000076293945" hidden="0" customWidth="1"/>
@@ -1980,11 +1979,11 @@
         <x:v>Accounts</x:v>
       </x:c>
       <x:c r="B4" s="18" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C4" s="18" t="n">
-        <x:f>COUNTA('Accounts'!$A$4:$A$23)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTA('Accounts'!$A$4:$A$25)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:f>IF(B4=C4,"PASS","FAIL")</x:f>
@@ -1996,11 +1995,11 @@
         <x:v>Profiles</x:v>
       </x:c>
       <x:c r="B5" s="18" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="18" t="n">
-        <x:f>COUNTA('Profiles'!$A$4:$A$23)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTA('Profiles'!$A$4:$A$25)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:f>IF(B5=C5,"PASS","FAIL")</x:f>
@@ -2153,7 +2152,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18" t="str">
-        <x:v>Production secret cells</x:v>
+        <x:v>Credential value cells</x:v>
       </x:c>
       <x:c r="B15" s="18" t="n">
         <x:v>0</x:v>
@@ -2176,7 +2175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3dd2aea1bdf4ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09190013ddff411c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2226,11 +2225,11 @@
         <x:v>Accounts</x:v>
       </x:c>
       <x:c r="B4" s="18" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C4" s="18" t="n">
         <x:f>'Validation Reconciliation'!C4</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:f>IF(B4=C4,"PASS","FAIL")</x:f>
@@ -2311,7 +2310,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb83f031d46724ca5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6014d4583134c1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2320,12 +2319,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16.670000076293945" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2336,7 +2334,6 @@
       <x:c r="C1" s="15"/>
       <x:c r="D1" s="15"/>
       <x:c r="E1" s="15"/>
-      <x:c r="F1" s="15"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="16" t="str">
@@ -2346,7 +2343,6 @@
       <x:c r="C2" s="16"/>
       <x:c r="D2" s="16"/>
       <x:c r="E2" s="16"/>
-      <x:c r="F2" s="16"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="17" t="str">
@@ -2356,16 +2352,13 @@
         <x:v>Hidden Auth Email</x:v>
       </x:c>
       <x:c r="C3" s="17" t="str">
-        <x:v>Role</x:v>
+        <x:v>Role Grants</x:v>
       </x:c>
       <x:c r="D3" s="17" t="str">
         <x:v>User ID</x:v>
       </x:c>
       <x:c r="E3" s="17" t="str">
-        <x:v>Local QA Password</x:v>
-      </x:c>
-      <x:c r="F3" s="17" t="str">
-        <x:v>Password Guard</x:v>
+        <x:v>Credential Source</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2382,10 +2375,7 @@
         <x:v>a1000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2402,10 +2392,7 @@
         <x:v>a1000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F5" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2422,10 +2409,7 @@
         <x:v>a1000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F6" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2442,10 +2426,7 @@
         <x:v>a1000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F7" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2462,10 +2443,7 @@
         <x:v>a1000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F8" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2482,10 +2460,7 @@
         <x:v>a2000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F9" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2502,10 +2477,7 @@
         <x:v>a2000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F10" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2522,10 +2494,7 @@
         <x:v>a2000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F11" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2542,10 +2511,7 @@
         <x:v>a2000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F12" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2562,10 +2528,7 @@
         <x:v>a2000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F13" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2582,10 +2545,7 @@
         <x:v>a3000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F14" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2602,10 +2562,7 @@
         <x:v>a3000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F15" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2622,10 +2579,7 @@
         <x:v>a3000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F16" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2642,10 +2596,7 @@
         <x:v>a3000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F17" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2662,10 +2613,7 @@
         <x:v>a3000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F18" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2682,10 +2630,7 @@
         <x:v>a4000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F19" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2702,10 +2647,7 @@
         <x:v>a4000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F20" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2722,10 +2664,7 @@
         <x:v>a4000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F21" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2742,10 +2681,7 @@
         <x:v>a4000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F22" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2762,20 +2698,51 @@
         <x:v>a4000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>Password</x:v>
-      </x:c>
-      <x:c r="F23" s="18" t="str">
-        <x:v>LOCAL_ONLY</x:v>
+        <x:v>ENV_REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="18" t="str">
+        <x:v>multi-role</x:v>
+      </x:c>
+      <x:c r="B24" s="18" t="str">
+        <x:v>multi-role@local.saqeel.test</x:v>
+      </x:c>
+      <x:c r="C24" s="18" t="str">
+        <x:v>planner + supervisor</x:v>
+      </x:c>
+      <x:c r="D24" s="18" t="str">
+        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="E24" s="18" t="str">
+        <x:v>ENV_REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="18" t="str">
+        <x:v>no-workspace</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>no-workspace@local.saqeel.test</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
+        <x:v>none (refusal case)</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str">
+        <x:v>a6000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="str">
+        <x:v>ENV_REQUIRED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f2dca1d7f624ec8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d83659e6f734089"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2785,7 +2752,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
@@ -3232,6 +3199,42 @@
         <x:v>active</x:v>
       </x:c>
     </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="18" t="str">
+        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="B24" s="18" t="str">
+        <x:v>multi-role</x:v>
+      </x:c>
+      <x:c r="C24" s="18" t="str">
+        <x:v>ضابط تخطيط ومراجعة تجريبي</x:v>
+      </x:c>
+      <x:c r="D24" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E24" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F24" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="18" t="str">
+        <x:v>a6000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>no-workspace</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
+        <x:v>مستخدم بلا مساحة عمل تجريبي</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str"/>
+      <x:c r="E25" s="18" t="str"/>
+      <x:c r="F25" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -3239,7 +3242,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce0b74f9ce44418"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd883165f814185"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3466,7 +3469,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a638520b4954698"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd050f50ca0ea4d20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3672,7 +3675,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3098be215a64ae6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bf9563f5542b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3857,7 +3860,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b6fd18f8ce490c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c1ba9b5fb24dbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4042,7 +4045,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72d9f2dca7634452"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702f8827a9304cd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4126,7 +4129,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b58342f25724f3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27eefd159bdc46f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4395,7 +4398,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb4cd6ae57c34e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c96af435f8459c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(uat): normalize governed identities
</commit_message>
<xml_diff>
--- a/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
+++ b/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="Rc94a930d94e74d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="Rcf86e6669bfa4898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="R4be72473a09147d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="R72c1ce6851f34a12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="Rd9fa693efc0c4dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="R88dbd92e23ae4d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="Rf22c1128ace64030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="R261e0bd7c5f8495f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R441d130d4dc342b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="Rb8226e95fb5d4f8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="R5b1a831b8ea04dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R18a4068ec0e54ea4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="Rd5585572708242ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="R8b62ffb6494147ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="Rf604819390f64536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="Re8d240c01e3d4a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="R3c56eb7f14b14a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="Raa416988ca584d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="R359d009e64724865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="Rbe39af2db21947c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="Reb3ab03b2e8e40b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="R5249228aeb58427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="R3e6493fd73524860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="R910d7e68eefe4824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="R6c6c071ac1264952"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R232496e8907f4bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="R9d153eb3a6da4253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="Rf187bb1c5f53472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R7b62cb5593754ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="R96ccd997583742ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="Rca847527fab94861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="R50f64a7929c640f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="R4569a2c7c1354b99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="R8aeeef58224f4795"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -373,8 +373,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TAccounts" displayName="TAccounts" ref="A3:E25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:E25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TAccounts" displayName="TAccounts" ref="A3:E50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:E50"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Username"/>
     <x:tableColumn id="2" name="Hidden Auth Email"/>
@@ -387,8 +387,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TProfiles" displayName="TProfiles" ref="A3:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A3:F25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TProfiles" displayName="TProfiles" ref="A3:F50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:F50"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="User ID"/>
     <x:tableColumn id="2" name="Username"/>
@@ -823,7 +823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re52dbd542a6c4958"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2ce4b2b1d14fb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -987,7 +987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48902a7d58e447b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1bcaef0625c4854"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1126,7 +1126,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e3466ada3c94389"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94839658f7504e17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1350,7 +1350,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e7693d0c0cd41e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8d7b24ff8c41b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1577,7 +1577,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13bc69a397f74d99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11785ab1a95548b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1737,7 +1737,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954ad43bdd244055"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c23bb4abc574d16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1748,7 +1748,7 @@
   <x:cols>
     <x:col min="1" max="1" width="6.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="21.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.4399995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1790,7 +1790,7 @@
         <x:v>Environment</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>Guard loopback + production refusal</x:v>
+        <x:v>Guard approved non-production target + production refusal</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>n/a</x:v>
@@ -1818,7 +1818,7 @@
         <x:v>Auth users</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>Upsert 22 deterministic local identities</x:v>
+        <x:v>Reconcile 47 deterministic UAT identities</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>15</x:v>
@@ -1929,7 +1929,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f31b32a3fae4019"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4cebafdef343cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1979,11 +1979,11 @@
         <x:v>Accounts</x:v>
       </x:c>
       <x:c r="B4" s="18" t="n">
-        <x:v>22</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="18" t="n">
-        <x:f>COUNTA('Accounts'!$A$4:$A$25)</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTA('Accounts'!$A$4:$A$50)</x:f>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:f>IF(B4=C4,"PASS","FAIL")</x:f>
@@ -1995,11 +1995,11 @@
         <x:v>Profiles</x:v>
       </x:c>
       <x:c r="B5" s="18" t="n">
-        <x:v>22</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C5" s="18" t="n">
-        <x:f>COUNTA('Profiles'!$A$4:$A$25)</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTA('Profiles'!$A$4:$A$50)</x:f>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:f>IF(B5=C5,"PASS","FAIL")</x:f>
@@ -2175,7 +2175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09190013ddff411c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01313c037b69425a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2200,7 +2200,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="16" t="str">
-        <x:v>Executive reconciliation for the local-only governed package.</x:v>
+        <x:v>Executive reconciliation for the governed non-production package.</x:v>
       </x:c>
       <x:c r="B2" s="16"/>
       <x:c r="C2" s="16"/>
@@ -2225,11 +2225,11 @@
         <x:v>Accounts</x:v>
       </x:c>
       <x:c r="B4" s="18" t="n">
-        <x:v>22</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="18" t="n">
         <x:f>'Validation Reconciliation'!C4</x:f>
-        <x:v>22</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:f>IF(B4=C4,"PASS","FAIL")</x:f>
@@ -2310,7 +2310,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6014d4583134c1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc67bdf212b484c64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2320,10 +2320,10 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20.559999465942383" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2366,7 +2366,7 @@
         <x:v>admin1</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
-        <x:v>admin1@local.saqeel.test</x:v>
+        <x:v>admin1@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
         <x:v>admin</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>a1000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2383,7 +2383,7 @@
         <x:v>admin2</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
-        <x:v>admin2@local.saqeel.test</x:v>
+        <x:v>admin2@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
         <x:v>admin</x:v>
@@ -2392,7 +2392,7 @@
         <x:v>a1000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2400,7 +2400,7 @@
         <x:v>admin3</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
-        <x:v>admin3@local.saqeel.test</x:v>
+        <x:v>admin3@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
         <x:v>admin</x:v>
@@ -2409,7 +2409,7 @@
         <x:v>a1000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2417,7 +2417,7 @@
         <x:v>admin4</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
-        <x:v>admin4@local.saqeel.test</x:v>
+        <x:v>admin4@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
         <x:v>admin</x:v>
@@ -2426,7 +2426,7 @@
         <x:v>a1000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2434,7 +2434,7 @@
         <x:v>admin5</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>admin5@local.saqeel.test</x:v>
+        <x:v>admin5@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
         <x:v>admin</x:v>
@@ -2443,7 +2443,7 @@
         <x:v>a1000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2451,7 +2451,7 @@
         <x:v>planner1</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
-        <x:v>planner1@local.saqeel.test</x:v>
+        <x:v>planner1@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
         <x:v>planner</x:v>
@@ -2460,7 +2460,7 @@
         <x:v>a2000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2468,7 +2468,7 @@
         <x:v>planner2</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>planner2@local.saqeel.test</x:v>
+        <x:v>planner2@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>planner</x:v>
@@ -2477,7 +2477,7 @@
         <x:v>a2000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2485,7 +2485,7 @@
         <x:v>planner3</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
-        <x:v>planner3@local.saqeel.test</x:v>
+        <x:v>planner3@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
         <x:v>planner</x:v>
@@ -2494,7 +2494,7 @@
         <x:v>a2000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2502,7 +2502,7 @@
         <x:v>planner4</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
-        <x:v>planner4@local.saqeel.test</x:v>
+        <x:v>planner4@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
         <x:v>planner</x:v>
@@ -2511,7 +2511,7 @@
         <x:v>a2000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2519,7 +2519,7 @@
         <x:v>planner5</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>planner5@local.saqeel.test</x:v>
+        <x:v>planner5@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
         <x:v>planner</x:v>
@@ -2528,7 +2528,7 @@
         <x:v>a2000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2536,7 +2536,7 @@
         <x:v>supervisor1</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
-        <x:v>supervisor1@local.saqeel.test</x:v>
+        <x:v>supervisor1@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
         <x:v>supervisor</x:v>
@@ -2545,7 +2545,7 @@
         <x:v>a3000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2553,7 +2553,7 @@
         <x:v>supervisor2</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>supervisor2@local.saqeel.test</x:v>
+        <x:v>supervisor2@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
         <x:v>supervisor</x:v>
@@ -2562,7 +2562,7 @@
         <x:v>a3000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2570,7 +2570,7 @@
         <x:v>supervisor3</x:v>
       </x:c>
       <x:c r="B16" s="18" t="str">
-        <x:v>supervisor3@local.saqeel.test</x:v>
+        <x:v>supervisor3@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C16" s="18" t="str">
         <x:v>supervisor</x:v>
@@ -2579,7 +2579,7 @@
         <x:v>a3000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2587,7 +2587,7 @@
         <x:v>supervisor4</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>supervisor4@local.saqeel.test</x:v>
+        <x:v>supervisor4@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
         <x:v>supervisor</x:v>
@@ -2596,7 +2596,7 @@
         <x:v>a3000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2604,7 +2604,7 @@
         <x:v>supervisor5</x:v>
       </x:c>
       <x:c r="B18" s="18" t="str">
-        <x:v>supervisor5@local.saqeel.test</x:v>
+        <x:v>supervisor5@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C18" s="18" t="str">
         <x:v>supervisor</x:v>
@@ -2613,7 +2613,7 @@
         <x:v>a3000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2621,7 +2621,7 @@
         <x:v>inspector1</x:v>
       </x:c>
       <x:c r="B19" s="18" t="str">
-        <x:v>inspector1@local.saqeel.test</x:v>
+        <x:v>inspector1@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C19" s="18" t="str">
         <x:v>inspector</x:v>
@@ -2630,7 +2630,7 @@
         <x:v>a4000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2638,7 +2638,7 @@
         <x:v>inspector2</x:v>
       </x:c>
       <x:c r="B20" s="18" t="str">
-        <x:v>inspector2@local.saqeel.test</x:v>
+        <x:v>inspector2@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C20" s="18" t="str">
         <x:v>inspector</x:v>
@@ -2647,7 +2647,7 @@
         <x:v>a4000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2655,7 +2655,7 @@
         <x:v>inspector3</x:v>
       </x:c>
       <x:c r="B21" s="18" t="str">
-        <x:v>inspector3@local.saqeel.test</x:v>
+        <x:v>inspector3@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C21" s="18" t="str">
         <x:v>inspector</x:v>
@@ -2664,7 +2664,7 @@
         <x:v>a4000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2672,7 +2672,7 @@
         <x:v>inspector4</x:v>
       </x:c>
       <x:c r="B22" s="18" t="str">
-        <x:v>inspector4@local.saqeel.test</x:v>
+        <x:v>inspector4@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C22" s="18" t="str">
         <x:v>inspector</x:v>
@@ -2681,7 +2681,7 @@
         <x:v>a4000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2689,7 +2689,7 @@
         <x:v>inspector5</x:v>
       </x:c>
       <x:c r="B23" s="18" t="str">
-        <x:v>inspector5@local.saqeel.test</x:v>
+        <x:v>inspector5@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C23" s="18" t="str">
         <x:v>inspector</x:v>
@@ -2698,41 +2698,466 @@
         <x:v>a4000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="18" t="str">
-        <x:v>multi-role</x:v>
+        <x:v>inspector6</x:v>
       </x:c>
       <x:c r="B24" s="18" t="str">
-        <x:v>multi-role@local.saqeel.test</x:v>
+        <x:v>inspector6@mim.gov.sa</x:v>
       </x:c>
       <x:c r="C24" s="18" t="str">
-        <x:v>planner + supervisor</x:v>
+        <x:v>inspector</x:v>
       </x:c>
       <x:c r="D24" s="18" t="str">
-        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+        <x:v>a4000000-0000-4000-8000-000000000006</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18" t="str">
+        <x:v>inspector7</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>inspector7@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000007</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="18" t="str">
+        <x:v>inspector8</x:v>
+      </x:c>
+      <x:c r="B26" s="18" t="str">
+        <x:v>inspector8@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C26" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D26" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000008</x:v>
+      </x:c>
+      <x:c r="E26" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="18" t="str">
+        <x:v>inspector9</x:v>
+      </x:c>
+      <x:c r="B27" s="18" t="str">
+        <x:v>inspector9@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C27" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D27" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000009</x:v>
+      </x:c>
+      <x:c r="E27" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="18" t="str">
+        <x:v>inspector10</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>inspector10@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C28" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D28" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000010</x:v>
+      </x:c>
+      <x:c r="E28" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="18" t="str">
+        <x:v>inspector11</x:v>
+      </x:c>
+      <x:c r="B29" s="18" t="str">
+        <x:v>inspector11@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C29" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D29" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000011</x:v>
+      </x:c>
+      <x:c r="E29" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="18" t="str">
+        <x:v>inspector12</x:v>
+      </x:c>
+      <x:c r="B30" s="18" t="str">
+        <x:v>inspector12@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C30" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D30" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000012</x:v>
+      </x:c>
+      <x:c r="E30" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="18" t="str">
+        <x:v>inspector13</x:v>
+      </x:c>
+      <x:c r="B31" s="18" t="str">
+        <x:v>inspector13@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C31" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D31" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000013</x:v>
+      </x:c>
+      <x:c r="E31" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="18" t="str">
+        <x:v>inspector14</x:v>
+      </x:c>
+      <x:c r="B32" s="18" t="str">
+        <x:v>inspector14@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C32" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D32" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000014</x:v>
+      </x:c>
+      <x:c r="E32" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="18" t="str">
+        <x:v>inspector15</x:v>
+      </x:c>
+      <x:c r="B33" s="18" t="str">
+        <x:v>inspector15@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C33" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D33" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000015</x:v>
+      </x:c>
+      <x:c r="E33" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="18" t="str">
+        <x:v>inspector16</x:v>
+      </x:c>
+      <x:c r="B34" s="18" t="str">
+        <x:v>inspector16@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C34" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D34" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000016</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="18" t="str">
+        <x:v>inspector17</x:v>
+      </x:c>
+      <x:c r="B35" s="18" t="str">
+        <x:v>inspector17@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C35" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D35" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000017</x:v>
+      </x:c>
+      <x:c r="E35" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="18" t="str">
+        <x:v>inspector18</x:v>
+      </x:c>
+      <x:c r="B36" s="18" t="str">
+        <x:v>inspector18@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C36" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D36" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000018</x:v>
+      </x:c>
+      <x:c r="E36" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="18" t="str">
+        <x:v>inspector19</x:v>
+      </x:c>
+      <x:c r="B37" s="18" t="str">
+        <x:v>inspector19@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C37" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D37" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000019</x:v>
+      </x:c>
+      <x:c r="E37" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="18" t="str">
+        <x:v>inspector20</x:v>
+      </x:c>
+      <x:c r="B38" s="18" t="str">
+        <x:v>inspector20@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C38" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D38" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000020</x:v>
+      </x:c>
+      <x:c r="E38" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="18" t="str">
+        <x:v>inspector21</x:v>
+      </x:c>
+      <x:c r="B39" s="18" t="str">
+        <x:v>inspector21@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C39" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D39" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000021</x:v>
+      </x:c>
+      <x:c r="E39" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="18" t="str">
+        <x:v>inspector22</x:v>
+      </x:c>
+      <x:c r="B40" s="18" t="str">
+        <x:v>inspector22@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C40" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D40" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000022</x:v>
+      </x:c>
+      <x:c r="E40" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="18" t="str">
+        <x:v>inspector23</x:v>
+      </x:c>
+      <x:c r="B41" s="18" t="str">
+        <x:v>inspector23@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C41" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D41" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000023</x:v>
+      </x:c>
+      <x:c r="E41" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="18" t="str">
+        <x:v>inspector24</x:v>
+      </x:c>
+      <x:c r="B42" s="18" t="str">
+        <x:v>inspector24@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C42" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D42" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000024</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="18" t="str">
+        <x:v>inspector25</x:v>
+      </x:c>
+      <x:c r="B43" s="18" t="str">
+        <x:v>inspector25@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C43" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000025</x:v>
+      </x:c>
+      <x:c r="E43" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="18" t="str">
+        <x:v>inspector26</x:v>
+      </x:c>
+      <x:c r="B44" s="18" t="str">
+        <x:v>inspector26@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C44" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000026</x:v>
+      </x:c>
+      <x:c r="E44" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="18" t="str">
+        <x:v>inspector27</x:v>
+      </x:c>
+      <x:c r="B45" s="18" t="str">
+        <x:v>inspector27@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C45" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D45" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000027</x:v>
+      </x:c>
+      <x:c r="E45" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="18" t="str">
+        <x:v>inspector28</x:v>
+      </x:c>
+      <x:c r="B46" s="18" t="str">
+        <x:v>inspector28@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C46" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D46" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000028</x:v>
+      </x:c>
+      <x:c r="E46" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="18" t="str">
+        <x:v>inspector29</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="str">
+        <x:v>inspector29@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C47" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D47" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000029</x:v>
+      </x:c>
+      <x:c r="E47" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="18" t="str">
+        <x:v>inspector30</x:v>
+      </x:c>
+      <x:c r="B48" s="18" t="str">
+        <x:v>inspector30@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C48" s="18" t="str">
+        <x:v>inspector</x:v>
+      </x:c>
+      <x:c r="D48" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000030</x:v>
+      </x:c>
+      <x:c r="E48" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="18" t="str">
+        <x:v>multi-role</x:v>
+      </x:c>
+      <x:c r="B49" s="18" t="str">
+        <x:v>multi-role@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C49" s="18" t="str">
+        <x:v>planner + supervisor</x:v>
+      </x:c>
+      <x:c r="D49" s="18" t="str">
+        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="E49" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="18" t="str">
         <x:v>no-workspace</x:v>
       </x:c>
-      <x:c r="B25" s="18" t="str">
-        <x:v>no-workspace@local.saqeel.test</x:v>
-      </x:c>
-      <x:c r="C25" s="18" t="str">
+      <x:c r="B50" s="18" t="str">
+        <x:v>no-workspace@mim.gov.sa</x:v>
+      </x:c>
+      <x:c r="C50" s="18" t="str">
         <x:v>none (refusal case)</x:v>
       </x:c>
-      <x:c r="D25" s="18" t="str">
+      <x:c r="D50" s="18" t="str">
         <x:v>a6000000-0000-4000-8000-000000000001</x:v>
       </x:c>
-      <x:c r="E25" s="18" t="str">
-        <x:v>ENV_REQUIRED</x:v>
+      <x:c r="E50" s="18" t="str">
+        <x:v>SAQEEL_UAT_PASSWORD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2742,7 +3167,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d83659e6f734089"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4379ea3dff604522"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3201,13 +3626,13 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="18" t="str">
-        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+        <x:v>a4000000-0000-4000-8000-000000000006</x:v>
       </x:c>
       <x:c r="B24" s="18" t="str">
-        <x:v>multi-role</x:v>
+        <x:v>inspector6</x:v>
       </x:c>
       <x:c r="C24" s="18" t="str">
-        <x:v>ضابط تخطيط ومراجعة تجريبي</x:v>
+        <x:v>Synthetic Inspector 06</x:v>
       </x:c>
       <x:c r="D24" s="18" t="str">
         <x:v>Riyadh</x:v>
@@ -3221,17 +3646,517 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000007</x:v>
+      </x:c>
+      <x:c r="B25" s="18" t="str">
+        <x:v>inspector7</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
+        <x:v>Synthetic Inspector 07</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str">
+        <x:v>Eastern Province</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F25" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000008</x:v>
+      </x:c>
+      <x:c r="B26" s="18" t="str">
+        <x:v>inspector8</x:v>
+      </x:c>
+      <x:c r="C26" s="18" t="str">
+        <x:v>Synthetic Inspector 08</x:v>
+      </x:c>
+      <x:c r="D26" s="18" t="str">
+        <x:v>Makkah</x:v>
+      </x:c>
+      <x:c r="E26" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F26" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000009</x:v>
+      </x:c>
+      <x:c r="B27" s="18" t="str">
+        <x:v>inspector9</x:v>
+      </x:c>
+      <x:c r="C27" s="18" t="str">
+        <x:v>Synthetic Inspector 09</x:v>
+      </x:c>
+      <x:c r="D27" s="18" t="str">
+        <x:v>Madinah</x:v>
+      </x:c>
+      <x:c r="E27" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F27" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000010</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>inspector10</x:v>
+      </x:c>
+      <x:c r="C28" s="18" t="str">
+        <x:v>Synthetic Inspector 10</x:v>
+      </x:c>
+      <x:c r="D28" s="18" t="str">
+        <x:v>Qassim</x:v>
+      </x:c>
+      <x:c r="E28" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F28" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000011</x:v>
+      </x:c>
+      <x:c r="B29" s="18" t="str">
+        <x:v>inspector11</x:v>
+      </x:c>
+      <x:c r="C29" s="18" t="str">
+        <x:v>Synthetic Inspector 11</x:v>
+      </x:c>
+      <x:c r="D29" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E29" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F29" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000012</x:v>
+      </x:c>
+      <x:c r="B30" s="18" t="str">
+        <x:v>inspector12</x:v>
+      </x:c>
+      <x:c r="C30" s="18" t="str">
+        <x:v>Synthetic Inspector 12</x:v>
+      </x:c>
+      <x:c r="D30" s="18" t="str">
+        <x:v>Eastern Province</x:v>
+      </x:c>
+      <x:c r="E30" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F30" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000013</x:v>
+      </x:c>
+      <x:c r="B31" s="18" t="str">
+        <x:v>inspector13</x:v>
+      </x:c>
+      <x:c r="C31" s="18" t="str">
+        <x:v>Synthetic Inspector 13</x:v>
+      </x:c>
+      <x:c r="D31" s="18" t="str">
+        <x:v>Makkah</x:v>
+      </x:c>
+      <x:c r="E31" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F31" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000014</x:v>
+      </x:c>
+      <x:c r="B32" s="18" t="str">
+        <x:v>inspector14</x:v>
+      </x:c>
+      <x:c r="C32" s="18" t="str">
+        <x:v>Synthetic Inspector 14</x:v>
+      </x:c>
+      <x:c r="D32" s="18" t="str">
+        <x:v>Madinah</x:v>
+      </x:c>
+      <x:c r="E32" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F32" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000015</x:v>
+      </x:c>
+      <x:c r="B33" s="18" t="str">
+        <x:v>inspector15</x:v>
+      </x:c>
+      <x:c r="C33" s="18" t="str">
+        <x:v>Synthetic Inspector 15</x:v>
+      </x:c>
+      <x:c r="D33" s="18" t="str">
+        <x:v>Qassim</x:v>
+      </x:c>
+      <x:c r="E33" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F33" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000016</x:v>
+      </x:c>
+      <x:c r="B34" s="18" t="str">
+        <x:v>inspector16</x:v>
+      </x:c>
+      <x:c r="C34" s="18" t="str">
+        <x:v>Synthetic Inspector 16</x:v>
+      </x:c>
+      <x:c r="D34" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F34" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000017</x:v>
+      </x:c>
+      <x:c r="B35" s="18" t="str">
+        <x:v>inspector17</x:v>
+      </x:c>
+      <x:c r="C35" s="18" t="str">
+        <x:v>Synthetic Inspector 17</x:v>
+      </x:c>
+      <x:c r="D35" s="18" t="str">
+        <x:v>Eastern Province</x:v>
+      </x:c>
+      <x:c r="E35" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F35" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000018</x:v>
+      </x:c>
+      <x:c r="B36" s="18" t="str">
+        <x:v>inspector18</x:v>
+      </x:c>
+      <x:c r="C36" s="18" t="str">
+        <x:v>Synthetic Inspector 18</x:v>
+      </x:c>
+      <x:c r="D36" s="18" t="str">
+        <x:v>Makkah</x:v>
+      </x:c>
+      <x:c r="E36" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F36" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000019</x:v>
+      </x:c>
+      <x:c r="B37" s="18" t="str">
+        <x:v>inspector19</x:v>
+      </x:c>
+      <x:c r="C37" s="18" t="str">
+        <x:v>Synthetic Inspector 19</x:v>
+      </x:c>
+      <x:c r="D37" s="18" t="str">
+        <x:v>Madinah</x:v>
+      </x:c>
+      <x:c r="E37" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F37" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000020</x:v>
+      </x:c>
+      <x:c r="B38" s="18" t="str">
+        <x:v>inspector20</x:v>
+      </x:c>
+      <x:c r="C38" s="18" t="str">
+        <x:v>Synthetic Inspector 20</x:v>
+      </x:c>
+      <x:c r="D38" s="18" t="str">
+        <x:v>Qassim</x:v>
+      </x:c>
+      <x:c r="E38" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F38" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000021</x:v>
+      </x:c>
+      <x:c r="B39" s="18" t="str">
+        <x:v>inspector21</x:v>
+      </x:c>
+      <x:c r="C39" s="18" t="str">
+        <x:v>Synthetic Inspector 21</x:v>
+      </x:c>
+      <x:c r="D39" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E39" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F39" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000022</x:v>
+      </x:c>
+      <x:c r="B40" s="18" t="str">
+        <x:v>inspector22</x:v>
+      </x:c>
+      <x:c r="C40" s="18" t="str">
+        <x:v>Synthetic Inspector 22</x:v>
+      </x:c>
+      <x:c r="D40" s="18" t="str">
+        <x:v>Eastern Province</x:v>
+      </x:c>
+      <x:c r="E40" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F40" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000023</x:v>
+      </x:c>
+      <x:c r="B41" s="18" t="str">
+        <x:v>inspector23</x:v>
+      </x:c>
+      <x:c r="C41" s="18" t="str">
+        <x:v>Synthetic Inspector 23</x:v>
+      </x:c>
+      <x:c r="D41" s="18" t="str">
+        <x:v>Makkah</x:v>
+      </x:c>
+      <x:c r="E41" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F41" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000024</x:v>
+      </x:c>
+      <x:c r="B42" s="18" t="str">
+        <x:v>inspector24</x:v>
+      </x:c>
+      <x:c r="C42" s="18" t="str">
+        <x:v>Synthetic Inspector 24</x:v>
+      </x:c>
+      <x:c r="D42" s="18" t="str">
+        <x:v>Madinah</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F42" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000025</x:v>
+      </x:c>
+      <x:c r="B43" s="18" t="str">
+        <x:v>inspector25</x:v>
+      </x:c>
+      <x:c r="C43" s="18" t="str">
+        <x:v>Synthetic Inspector 25</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="str">
+        <x:v>Qassim</x:v>
+      </x:c>
+      <x:c r="E43" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F43" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000026</x:v>
+      </x:c>
+      <x:c r="B44" s="18" t="str">
+        <x:v>inspector26</x:v>
+      </x:c>
+      <x:c r="C44" s="18" t="str">
+        <x:v>Synthetic Inspector 26</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E44" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F44" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000027</x:v>
+      </x:c>
+      <x:c r="B45" s="18" t="str">
+        <x:v>inspector27</x:v>
+      </x:c>
+      <x:c r="C45" s="18" t="str">
+        <x:v>Synthetic Inspector 27</x:v>
+      </x:c>
+      <x:c r="D45" s="18" t="str">
+        <x:v>Eastern Province</x:v>
+      </x:c>
+      <x:c r="E45" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F45" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000028</x:v>
+      </x:c>
+      <x:c r="B46" s="18" t="str">
+        <x:v>inspector28</x:v>
+      </x:c>
+      <x:c r="C46" s="18" t="str">
+        <x:v>Synthetic Inspector 28</x:v>
+      </x:c>
+      <x:c r="D46" s="18" t="str">
+        <x:v>Makkah</x:v>
+      </x:c>
+      <x:c r="E46" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F46" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000029</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="str">
+        <x:v>inspector29</x:v>
+      </x:c>
+      <x:c r="C47" s="18" t="str">
+        <x:v>Synthetic Inspector 29</x:v>
+      </x:c>
+      <x:c r="D47" s="18" t="str">
+        <x:v>Madinah</x:v>
+      </x:c>
+      <x:c r="E47" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F47" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="18" t="str">
+        <x:v>a4000000-0000-4000-8000-000000000030</x:v>
+      </x:c>
+      <x:c r="B48" s="18" t="str">
+        <x:v>inspector30</x:v>
+      </x:c>
+      <x:c r="C48" s="18" t="str">
+        <x:v>Synthetic Inspector 30</x:v>
+      </x:c>
+      <x:c r="D48" s="18" t="str">
+        <x:v>Qassim</x:v>
+      </x:c>
+      <x:c r="E48" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F48" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="18" t="str">
+        <x:v>a5000000-0000-4000-8000-000000000001</x:v>
+      </x:c>
+      <x:c r="B49" s="18" t="str">
+        <x:v>multi-role</x:v>
+      </x:c>
+      <x:c r="C49" s="18" t="str">
+        <x:v>ضابط تخطيط ومراجعة تجريبي</x:v>
+      </x:c>
+      <x:c r="D49" s="18" t="str">
+        <x:v>Riyadh</x:v>
+      </x:c>
+      <x:c r="E49" s="18" t="str">
+        <x:v>regional</x:v>
+      </x:c>
+      <x:c r="F49" s="18" t="str">
+        <x:v>active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="18" t="str">
         <x:v>a6000000-0000-4000-8000-000000000001</x:v>
       </x:c>
-      <x:c r="B25" s="18" t="str">
+      <x:c r="B50" s="18" t="str">
         <x:v>no-workspace</x:v>
       </x:c>
-      <x:c r="C25" s="18" t="str">
+      <x:c r="C50" s="18" t="str">
         <x:v>مستخدم بلا مساحة عمل تجريبي</x:v>
       </x:c>
-      <x:c r="D25" s="18" t="str"/>
-      <x:c r="E25" s="18" t="str"/>
-      <x:c r="F25" s="18" t="str">
+      <x:c r="D50" s="18" t="str"/>
+      <x:c r="E50" s="18" t="str"/>
+      <x:c r="F50" s="18" t="str">
         <x:v>active</x:v>
       </x:c>
     </x:row>
@@ -3242,7 +4167,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd883165f814185"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra041655f80c843f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3469,7 +4394,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd050f50ca0ea4d20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb3742292a840c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3675,7 +4600,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365bf9563f5542b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cbb851b241e4721"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3860,7 +4785,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32c1ba9b5fb24dbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R697b3e6a47254baa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4045,7 +4970,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702f8827a9304cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re77aa3de405b4cf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4129,7 +5054,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27eefd159bdc46f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc243d8cf0ddf472e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4398,7 +5323,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c96af435f8459c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cf85fdc20e34a62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(uat): reuse governed cohort secret
</commit_message>
<xml_diff>
--- a/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
+++ b/outputs/019fbd0c-8368-7a72-819b-32653b4d1e65/SAQEEL_Local_Test_Data_Package.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="Raa416988ca584d11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="R359d009e64724865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="Rbe39af2db21947c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="Reb3ab03b2e8e40b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="R5249228aeb58427c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="R3e6493fd73524860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="R910d7e68eefe4824"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="R6c6c071ac1264952"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R232496e8907f4bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="R9d153eb3a6da4253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="Rf187bb1c5f53472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R7b62cb5593754ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="R96ccd997583742ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="Rca847527fab94861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="R50f64a7929c640f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="R4569a2c7c1354b99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="R8aeeef58224f4795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Controls" sheetId="1" r:id="R8fa8a3ac3285438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" r:id="R5246df52e6ff4be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="3" r:id="R7ec6a1ee4fb54812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Establishments" sheetId="4" r:id="Rdceaaef091b84457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="5" r:id="R6bc1c92f695f487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Packages Templates" sheetId="6" r:id="Rd932fc6d78af424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="7" r:id="Rf0e00b99a0a94106"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Plans" sheetId="8" r:id="Rce630709a2da4d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visits" sheetId="9" r:id="R45359f8400c84967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="10" r:id="R9175ca2386cc47f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inspection Data" sheetId="11" r:id="Rc5f4980a9db54d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Reports Evidence" sheetId="12" r:id="R7210dafe46e04c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Matrix" sheetId="13" r:id="Rffbd0d91519c4ad9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="14" r:id="R47a2d3be195740bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Order" sheetId="15" r:id="R8f13f212263f4231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Reconciliation" sheetId="16" r:id="R66128a4c72814bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Summary" sheetId="17" r:id="Rb97d049043ed4132"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -823,7 +823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2ce4b2b1d14fb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R330bdd66e5964938"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -987,7 +987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1bcaef0625c4854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref8f3d541efa4e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1126,7 +1126,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94839658f7504e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43fbc7dd90644fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1350,7 +1350,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8d7b24ff8c41b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd36f85e03b0642e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1577,7 +1577,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11785ab1a95548b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31dbcf21eb74443c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1737,7 +1737,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c23bb4abc574d16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree75192d8ed34686"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1929,7 +1929,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4cebafdef343cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R551c5aeea7af4aca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2175,7 +2175,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01313c037b69425a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf12c1ddcb3244639"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2310,7 +2310,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc67bdf212b484c64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a049cc1ab50485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2323,7 +2323,7 @@
     <x:col min="2" max="2" width="20.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28.219999313354492" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -2375,7 +2375,7 @@
         <x:v>a1000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2392,7 +2392,7 @@
         <x:v>a1000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2409,7 +2409,7 @@
         <x:v>a1000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2426,7 +2426,7 @@
         <x:v>a1000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2443,7 +2443,7 @@
         <x:v>a1000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2460,7 +2460,7 @@
         <x:v>a2000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2477,7 +2477,7 @@
         <x:v>a2000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2494,7 +2494,7 @@
         <x:v>a2000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2511,7 +2511,7 @@
         <x:v>a2000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2528,7 +2528,7 @@
         <x:v>a2000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2545,7 +2545,7 @@
         <x:v>a3000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2562,7 +2562,7 @@
         <x:v>a3000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2579,7 +2579,7 @@
         <x:v>a3000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2596,7 +2596,7 @@
         <x:v>a3000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2613,7 +2613,7 @@
         <x:v>a3000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2630,7 +2630,7 @@
         <x:v>a4000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2647,7 +2647,7 @@
         <x:v>a4000000-0000-4000-8000-000000000002</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2664,7 +2664,7 @@
         <x:v>a4000000-0000-4000-8000-000000000003</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2681,7 +2681,7 @@
         <x:v>a4000000-0000-4000-8000-000000000004</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2698,7 +2698,7 @@
         <x:v>a4000000-0000-4000-8000-000000000005</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -2715,7 +2715,7 @@
         <x:v>a4000000-0000-4000-8000-000000000006</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2732,7 +2732,7 @@
         <x:v>a4000000-0000-4000-8000-000000000007</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2749,7 +2749,7 @@
         <x:v>a4000000-0000-4000-8000-000000000008</x:v>
       </x:c>
       <x:c r="E26" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -2766,7 +2766,7 @@
         <x:v>a4000000-0000-4000-8000-000000000009</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2783,7 +2783,7 @@
         <x:v>a4000000-0000-4000-8000-000000000010</x:v>
       </x:c>
       <x:c r="E28" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2800,7 +2800,7 @@
         <x:v>a4000000-0000-4000-8000-000000000011</x:v>
       </x:c>
       <x:c r="E29" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2817,7 +2817,7 @@
         <x:v>a4000000-0000-4000-8000-000000000012</x:v>
       </x:c>
       <x:c r="E30" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2834,7 +2834,7 @@
         <x:v>a4000000-0000-4000-8000-000000000013</x:v>
       </x:c>
       <x:c r="E31" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2851,7 +2851,7 @@
         <x:v>a4000000-0000-4000-8000-000000000014</x:v>
       </x:c>
       <x:c r="E32" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2868,7 +2868,7 @@
         <x:v>a4000000-0000-4000-8000-000000000015</x:v>
       </x:c>
       <x:c r="E33" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2885,7 +2885,7 @@
         <x:v>a4000000-0000-4000-8000-000000000016</x:v>
       </x:c>
       <x:c r="E34" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2902,7 +2902,7 @@
         <x:v>a4000000-0000-4000-8000-000000000017</x:v>
       </x:c>
       <x:c r="E35" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2919,7 +2919,7 @@
         <x:v>a4000000-0000-4000-8000-000000000018</x:v>
       </x:c>
       <x:c r="E36" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2936,7 +2936,7 @@
         <x:v>a4000000-0000-4000-8000-000000000019</x:v>
       </x:c>
       <x:c r="E37" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2953,7 +2953,7 @@
         <x:v>a4000000-0000-4000-8000-000000000020</x:v>
       </x:c>
       <x:c r="E38" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2970,7 +2970,7 @@
         <x:v>a4000000-0000-4000-8000-000000000021</x:v>
       </x:c>
       <x:c r="E39" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2987,7 +2987,7 @@
         <x:v>a4000000-0000-4000-8000-000000000022</x:v>
       </x:c>
       <x:c r="E40" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3004,7 +3004,7 @@
         <x:v>a4000000-0000-4000-8000-000000000023</x:v>
       </x:c>
       <x:c r="E41" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3021,7 +3021,7 @@
         <x:v>a4000000-0000-4000-8000-000000000024</x:v>
       </x:c>
       <x:c r="E42" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -3038,7 +3038,7 @@
         <x:v>a4000000-0000-4000-8000-000000000025</x:v>
       </x:c>
       <x:c r="E43" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -3055,7 +3055,7 @@
         <x:v>a4000000-0000-4000-8000-000000000026</x:v>
       </x:c>
       <x:c r="E44" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3072,7 +3072,7 @@
         <x:v>a4000000-0000-4000-8000-000000000027</x:v>
       </x:c>
       <x:c r="E45" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3089,7 +3089,7 @@
         <x:v>a4000000-0000-4000-8000-000000000028</x:v>
       </x:c>
       <x:c r="E46" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -3106,7 +3106,7 @@
         <x:v>a4000000-0000-4000-8000-000000000029</x:v>
       </x:c>
       <x:c r="E47" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -3123,7 +3123,7 @@
         <x:v>a4000000-0000-4000-8000-000000000030</x:v>
       </x:c>
       <x:c r="E48" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -3140,7 +3140,7 @@
         <x:v>a5000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E49" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -3157,7 +3157,7 @@
         <x:v>a6000000-0000-4000-8000-000000000001</x:v>
       </x:c>
       <x:c r="E50" s="18" t="str">
-        <x:v>SAQEEL_UAT_PASSWORD</x:v>
+        <x:v>SAQEEL_CROSS_ROLE_PASSWORD</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3167,7 +3167,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4379ea3dff604522"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bc31898304845c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4167,7 +4167,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra041655f80c843f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abbd921d7784bb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4394,7 +4394,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb3742292a840c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6ee3e91c8014602"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4600,7 +4600,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cbb851b241e4721"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9163cbb18d9244a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4785,7 +4785,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R697b3e6a47254baa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R092e33ac6510455e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4970,7 +4970,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re77aa3de405b4cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca60894731d4ac0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5054,7 +5054,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc243d8cf0ddf472e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6164518d9694e9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5323,7 +5323,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cf85fdc20e34a62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d9f9b56ff540ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>